<commit_message>
Add August monthly meeting deck and set slow-task metric to >2 days
Set the Tesorio slow-task threshold to >2 days permanently (scripts + report).
Add a monthly meeting PowerPoint deck (Portal Uploads + Tesorio Tasks, August)
using the shared template's color scheme, and its generator script.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nn9QKEstPX9eZ4ngSPWHBW
</commit_message>
<xml_diff>
--- a/Tesorio_Tasks_Report_Aug_2026.xlsx
+++ b/Tesorio_Tasks_Report_Aug_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Tesorio Tasks Report" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data (calc)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Open &amp; In Progress" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Slow Tasks Aug - 26 (&gt;7d)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Slow Tasks Aug - 26 (&gt;2d)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8157,7 +8157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8171,7 +8171,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>Aug - 26 TASKS RESOLVED IN MORE THAN 7 DAYS</t>
+          <t>Aug - 26 TASKS RESOLVED IN MORE THAN 2 DAYS</t>
         </is>
       </c>
     </row>
@@ -8258,6 +8258,195 @@
       </c>
       <c r="F5" s="21">
         <f>(E5-D5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>INV00023786</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Alberto Mirón 🦅</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>46255.84363528797</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>46259.99149806406</v>
+      </c>
+      <c r="F6" s="21">
+        <f>(E6-D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>470261</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Marco Guadarrama</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>46255.8231754211</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>46258.97525643204</v>
+      </c>
+      <c r="F7" s="21">
+        <f>(E7-D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>INV00022697</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>URGENT</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Ana Paula De la Vega</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>46252.69255169145</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>46254.94319169327</v>
+      </c>
+      <c r="F8" s="21">
+        <f>(E8-D8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>INV00022437</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Roberto Vázquez</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>46252.70366985427</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>46254.9452245279</v>
+      </c>
+      <c r="F9" s="21">
+        <f>(E9-D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>INV00025652</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Alberto Mirón 🦅</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>46252.70975034301</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>46254.94638165123</v>
+      </c>
+      <c r="F10" s="21">
+        <f>(E10-D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>INV00023564</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>URGENT</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Paolet Ordóñez</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>46252.75321715503</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>46254.94682119416</v>
+      </c>
+      <c r="F11" s="21">
+        <f>(E11-D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>INV00025585</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Fernanda Sánchez</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>46252.78873059987</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>46254.94785228158</v>
+      </c>
+      <c r="F12" s="21">
+        <f>(E12-D12)</f>
         <v/>
       </c>
     </row>

</xml_diff>